<commit_message>
Extraction Xlsx Formations : WIP
</commit_message>
<xml_diff>
--- a/module/Formation/resources/formation_stats_export.xlsx
+++ b/module/Formation/resources/formation_stats_export.xlsx
@@ -13,12 +13,13 @@
     <sheet name="DATA_ENQ" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="EnquetesReponses" sheetId="4" state="visible" r:id="rId5"/>
     <sheet name="EnquetesCommentaires" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="LOG" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="DATA_DOCTORANT" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="LOG" sheetId="7" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId9"/>
-    <pivotCache cacheId="2" r:id="rId10"/>
+    <pivotCache cacheId="1" r:id="rId10"/>
+    <pivotCache cacheId="2" r:id="rId11"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -1123,7 +1124,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:T68"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="121.34"/>
@@ -1568,10 +1569,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:T5"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11.64"/>
-  </cols>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3"/>
@@ -1800,7 +1798,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H1002"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="53.38"/>
@@ -4866,7 +4864,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44.18"/>
   </cols>
@@ -4962,7 +4960,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34.36"/>
@@ -5019,4 +5017,22 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>